<commit_message>
feat: modernize schedules UI, improve duty grid layout, and cleanup unused components
</commit_message>
<xml_diff>
--- a/OgretmenNobetListesi.xlsx
+++ b/OgretmenNobetListesi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a149d352df2b778d/Desktop/Programlar/nobetci-asistan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="11_375A638456655E6C26E55EC8EEFA6E1DEB75A23E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69426724-ED9F-403E-95D0-87863AA10076}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="11_375A638456655E6C26E55EC8EEFA6E1DEB75A23E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{345FB915-2BB9-43F3-A541-B6D147786457}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -424,11 +424,6 @@
 ENGİN KAYSERİLİ</t>
   </si>
   <si>
-    <t>SEÇİL ARI
-ÖMER MURAT YILDIZ 
-MAHMUT DOĞRUYOL</t>
-  </si>
-  <si>
     <t>SERDAR SAVAŞ 
 HALİL AKÇAY</t>
   </si>
@@ -464,6 +459,10 @@
   <si>
     <t>HAKKI AKARSU 
 BİLAL ŞENTÜRK</t>
+  </si>
+  <si>
+    <t>ÖMER MURAT YILDIZ 
+MAHMUT DOĞRUYOL</t>
   </si>
 </sst>
 </file>
@@ -635,6 +634,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -654,9 +656,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -674,6 +673,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -972,35 +975,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
     </row>
     <row r="2" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="17"/>
       <c r="I2" s="2"/>
     </row>
     <row r="3" spans="1:9" ht="49.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13"/>
+      <c r="A3" s="14"/>
       <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
@@ -1028,23 +1031,23 @@
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="F4" s="18" t="s">
+      <c r="F4" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="G4" s="18" t="s">
-        <v>45</v>
+      <c r="G4" s="11" t="s">
+        <v>44</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>11</v>
@@ -1055,23 +1058,23 @@
       <c r="A5" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="G5" s="18" t="s">
-        <v>46</v>
+      <c r="F5" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>45</v>
       </c>
       <c r="H5" s="10" t="s">
         <v>13</v>
@@ -1085,20 +1088,20 @@
       <c r="B6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="F6" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="G6" s="18" t="s">
-        <v>47</v>
+      <c r="F6" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>46</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>16</v>
@@ -1109,26 +1112,26 @@
       <c r="A7" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="F7" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="G7" s="18" t="s">
-        <v>48</v>
-      </c>
-      <c r="H7" s="18" t="s">
-        <v>50</v>
+      <c r="F7" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>49</v>
       </c>
       <c r="I7" s="2"/>
     </row>
@@ -1139,20 +1142,20 @@
       <c r="B8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="11" t="s">
         <v>35</v>
       </c>
       <c r="E8" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="G8" s="18" t="s">
-        <v>49</v>
+      <c r="F8" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>48</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>21</v>
@@ -1160,17 +1163,17 @@
       <c r="I8" s="2"/>
     </row>
     <row r="9" spans="1:9" ht="132" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>